<commit_message>
QAQC'd 2023 Syn Sulfide Data
</commit_message>
<xml_diff>
--- a/Porewater/Sulfide/Synoptic_CB/2023/Previous Codes/Datasheets/COMPASS_Synoptic_H2S_Oct2023.xlsx
+++ b/Porewater/Sulfide/Synoptic_CB/2023/Previous Codes/Datasheets/COMPASS_Synoptic_H2S_Oct2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Biogeochemistry\People\Wilson (Steph)\Data\MicroPlate Data\Sulfide\Data\2023\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/synoptic-discrete-data/Porewater/Sulfide/Synoptic_CB/2023/Previous Codes/Datasheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58735480-8CA6-4016-9CAA-4F2B7C624370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{58735480-8CA6-4016-9CAA-4F2B7C624370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F67E6BBB-40B9-4E51-8F71-AB1F3BAFEF51}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="3" activeTab="6" xr2:uid="{98C59184-82FD-4ED3-93B6-F57DE327E822}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{98C59184-82FD-4ED3-93B6-F57DE327E822}"/>
   </bookViews>
   <sheets>
     <sheet name="Stds" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
     <sheet name="Plate6" sheetId="8" r:id="rId7"/>
     <sheet name="Plate7" sheetId="9" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -46,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="184">
   <si>
     <t>Plate 1</t>
   </si>
@@ -7647,486 +7644,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="STDs"/>
-      <sheetName val="Plate1"/>
-      <sheetName val="Plate2"/>
-      <sheetName val="Plate3"/>
-      <sheetName val="Plate4"/>
-      <sheetName val="Plate5"/>
-      <sheetName val="Plate6"/>
-      <sheetName val="Plate7"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="2">
-          <cell r="B2" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>0</v>
-          </cell>
-          <cell r="B3">
-            <v>5.2666666666666667E-2</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>5</v>
-          </cell>
-          <cell r="B4">
-            <v>0.17433333333333334</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>12.5</v>
-          </cell>
-          <cell r="B5">
-            <v>0.496</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>25</v>
-          </cell>
-          <cell r="B6">
-            <v>0.73466666666666669</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>50</v>
-          </cell>
-          <cell r="B7">
-            <v>1.2829999999999999</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>100</v>
-          </cell>
-          <cell r="B8">
-            <v>1.9710000000000001</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>0</v>
-          </cell>
-          <cell r="B14">
-            <v>5.2333333333333336E-2</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>5</v>
-          </cell>
-          <cell r="B15">
-            <v>0.18733333333333335</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>12.5</v>
-          </cell>
-          <cell r="B16">
-            <v>0.5665</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>25</v>
-          </cell>
-          <cell r="B17">
-            <v>0.66866666666666674</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18">
-            <v>50</v>
-          </cell>
-          <cell r="B18">
-            <v>1.23</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19">
-            <v>100</v>
-          </cell>
-          <cell r="B19">
-            <v>1.7130000000000001</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="B24" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25">
-            <v>0</v>
-          </cell>
-          <cell r="B25">
-            <v>5.1999999999999998E-2</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26">
-            <v>5</v>
-          </cell>
-          <cell r="B26">
-            <v>0.17733333333333334</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27">
-            <v>12.5</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28">
-            <v>25</v>
-          </cell>
-          <cell r="B28">
-            <v>0.57000000000000006</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29">
-            <v>50</v>
-          </cell>
-          <cell r="B29">
-            <v>1.0415000000000001</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30">
-            <v>100</v>
-          </cell>
-          <cell r="B30">
-            <v>1.6234999999999999</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31">
-            <v>100</v>
-          </cell>
-          <cell r="B31">
-            <v>1.5263333333333333</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32">
-            <v>100</v>
-          </cell>
-          <cell r="B32">
-            <v>1.5759999999999998</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="B35" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="A36">
-            <v>0</v>
-          </cell>
-          <cell r="B36">
-            <v>5.5E-2</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="A37">
-            <v>5</v>
-          </cell>
-          <cell r="B37">
-            <v>0.16633333333333333</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="A38">
-            <v>12.5</v>
-          </cell>
-          <cell r="B38">
-            <v>0.57450000000000001</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="A39">
-            <v>25</v>
-          </cell>
-          <cell r="B39">
-            <v>0.51600000000000001</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="A40">
-            <v>50</v>
-          </cell>
-          <cell r="B40">
-            <v>1.1335</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="A41">
-            <v>100</v>
-          </cell>
-          <cell r="B41">
-            <v>1.6326666666666665</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="A42">
-            <v>100</v>
-          </cell>
-          <cell r="B42">
-            <v>1.6503333333333334</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43">
-            <v>100</v>
-          </cell>
-          <cell r="B43">
-            <v>1.7290000000000001</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="B46" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="A47">
-            <v>0</v>
-          </cell>
-          <cell r="B47">
-            <v>5.5333333333333325E-2</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="A48">
-            <v>5</v>
-          </cell>
-          <cell r="B48">
-            <v>0.158</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="A49">
-            <v>12.5</v>
-          </cell>
-          <cell r="B49">
-            <v>0.36866666666666664</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="A50">
-            <v>25</v>
-          </cell>
-          <cell r="B50">
-            <v>0.65666666666666673</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="A51">
-            <v>50</v>
-          </cell>
-          <cell r="B51">
-            <v>1.0549999999999999</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="A52">
-            <v>100</v>
-          </cell>
-          <cell r="B52">
-            <v>1.7556666666666665</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="A53">
-            <v>100</v>
-          </cell>
-          <cell r="B53">
-            <v>1.6950000000000001</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="A54">
-            <v>100</v>
-          </cell>
-          <cell r="B54">
-            <v>1.766</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="B57" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="A58">
-            <v>0</v>
-          </cell>
-          <cell r="B58">
-            <v>5.4666666666666669E-2</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="A59">
-            <v>5</v>
-          </cell>
-          <cell r="B59">
-            <v>0.20099999999999998</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="A60">
-            <v>12.5</v>
-          </cell>
-          <cell r="B60">
-            <v>0.36499999999999999</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="A61">
-            <v>25</v>
-          </cell>
-          <cell r="B61">
-            <v>0.75049999999999994</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="A62">
-            <v>50</v>
-          </cell>
-          <cell r="B62">
-            <v>1.169</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="A63">
-            <v>100</v>
-          </cell>
-          <cell r="B63">
-            <v>1.85</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="A64">
-            <v>100</v>
-          </cell>
-          <cell r="B64">
-            <v>1.7309999999999999</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="A65">
-            <v>100</v>
-          </cell>
-          <cell r="B65">
-            <v>1.8503333333333334</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="B69" t="str">
-            <v>Avg Abs</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="A70">
-            <v>0</v>
-          </cell>
-          <cell r="B70">
-            <v>5.2666666666666667E-2</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="A71">
-            <v>5</v>
-          </cell>
-          <cell r="B71">
-            <v>0.19600000000000004</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="A72">
-            <v>12.5</v>
-          </cell>
-          <cell r="B72">
-            <v>0.36266666666666669</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="A73">
-            <v>25</v>
-          </cell>
-          <cell r="B73">
-            <v>0.62450000000000006</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="A74">
-            <v>50</v>
-          </cell>
-          <cell r="B74">
-            <v>0.99550000000000005</v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="A75">
-            <v>100</v>
-          </cell>
-          <cell r="B75">
-            <v>1.6895</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="A76">
-            <v>100</v>
-          </cell>
-          <cell r="B76">
-            <v>1.6336666666666666</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="A77">
-            <v>100</v>
-          </cell>
-          <cell r="B77">
-            <v>1.72</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8164,7 +7685,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -8270,7 +7791,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8412,7 +7933,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9677,6 +9198,9 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
+      <c r="N1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -10759,10 +10283,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A73A72-21F5-4C48-AA99-1574BF45D156}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>31</v>
       </c>
@@ -10802,8 +10326,11 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -10844,7 +10371,7 @@
         <v>1.7669999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -10885,7 +10412,7 @@
         <v>1.694</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -10926,7 +10453,7 @@
         <v>1.746</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -10967,7 +10494,7 @@
         <v>1.7989999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -11008,7 +10535,7 @@
         <v>0.82599999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -11049,7 +10576,7 @@
         <v>0.873</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -11090,7 +10617,7 @@
         <v>1.3320000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -11131,7 +10658,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -11172,7 +10699,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -11213,7 +10740,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -11254,7 +10781,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -11295,7 +10822,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -11336,7 +10863,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -11877,10 +11404,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81B2B8CB-2535-41F0-9219-545A28B891F6}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>30</v>
       </c>
@@ -11920,8 +11447,11 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -11962,7 +11492,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -12003,7 +11533,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -12044,7 +11574,7 @@
         <v>0.184</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -12085,7 +11615,7 @@
         <v>6.5000000000000002E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -12126,7 +11656,7 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -12167,7 +11697,7 @@
         <v>0.82599999999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -12208,7 +11738,7 @@
         <v>0.127</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -12249,7 +11779,7 @@
         <v>2.0379999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -12290,7 +11820,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -12331,7 +11861,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -12372,7 +11902,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -12413,7 +11943,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -12454,7 +11984,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -12995,10 +12525,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD39B94D-19CA-455E-A862-7EAF25E75130}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5">
         <v>1</v>
@@ -13036,8 +12566,11 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -13078,7 +12611,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -13119,7 +12652,7 @@
         <v>0.314</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -13160,7 +12693,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -13201,7 +12734,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -13242,7 +12775,7 @@
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -13283,7 +12816,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -13324,7 +12857,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -13365,7 +12898,7 @@
         <v>0.129</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -13406,7 +12939,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -13447,7 +12980,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -13488,7 +13021,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -13529,7 +13062,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -13570,7 +13103,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -14110,10 +13643,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{368D03D9-B8AC-4D1D-BDDB-1783FF67E978}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>32</v>
       </c>
@@ -14153,8 +13686,11 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -14195,7 +13731,7 @@
         <v>6.3E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -14236,7 +13772,7 @@
         <v>6.3E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -14277,7 +13813,7 @@
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -14318,7 +13854,7 @@
         <v>6.9000000000000006E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -14359,7 +13895,7 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -14400,7 +13936,7 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -14441,7 +13977,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -14482,7 +14018,7 @@
         <v>5.3999999999999999E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -14523,7 +14059,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -14564,7 +14100,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -14605,7 +14141,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -14646,7 +14182,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -14687,7 +14223,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -15227,10 +14763,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B3DB1D0-27C9-44CA-88D0-D985F5267C57}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>153</v>
       </c>
@@ -15270,8 +14806,11 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -15312,7 +14851,7 @@
         <v>6.8000000000000005E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -15353,7 +14892,7 @@
         <v>0.20399999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -15394,7 +14933,7 @@
         <v>0.76700000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -15435,7 +14974,7 @@
         <v>0.53200000000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -15476,7 +15015,7 @@
         <v>0.91400000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -15517,7 +15056,7 @@
         <v>0.63400000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -15558,7 +15097,7 @@
         <v>0.221</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -15599,7 +15138,7 @@
         <v>0.871</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -15640,7 +15179,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -15681,7 +15220,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -15722,7 +15261,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -15763,7 +15302,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -15804,7 +15343,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
@@ -16345,10 +15884,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA28CD24-68E0-4F84-82D5-CD6F695F78C4}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>178</v>
       </c>
@@ -16388,8 +15927,11 @@
       <c r="M1" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -16430,7 +15972,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -16471,7 +16013,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -16512,7 +16054,7 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
@@ -16553,7 +16095,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
@@ -16594,7 +16136,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -16635,7 +16177,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -16676,7 +16218,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -16717,7 +16259,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
@@ -16758,7 +16300,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -16793,7 +16335,7 @@
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
@@ -16828,7 +16370,7 @@
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -16857,7 +16399,7 @@
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -16886,7 +16428,7 @@
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>16</v>
       </c>

</xml_diff>